<commit_message>
Fase 184: ID de la llamada (CONN_ID) en los comentarios de la Encuesta de Mobilize (v1.73.0)
- Lector: CONN_ID opcional del archivo de encuesta, con aviso si falta; el
  teléfono sigue sin leerse. Migración: columna connId ('' por defecto).
- Lista de comentarios y Excel: columna "ID de llamada" (vacía si el
  archivo no la traía; sin cruce con el CDR). Plantilla y ficha regeneradas.
- Arreglo de la Fase 178: los meses de los paneles ya no se pisan entre
  fuentes (un mes con solo Encuesta no salía en el MES de Mobilize).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_ENCUESTA.xlsx
+++ b/server/plantillas/PLANTILLA_ENCUESTA.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -408,6 +408,7 @@
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -435,17 +436,20 @@
       <c r="H1" t="str">
         <v>VOICE_MESSAGE</v>
       </c>
+      <c r="I1" t="str">
+        <v>CONN_ID</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -644,9 +648,26 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>CONN_ID</v>
+      </c>
+      <c r="B16" t="str">
+        <v>No</v>
+      </c>
+      <c r="C16" t="str">
+        <v>ID de la llamada en Wolkvox (opcional). Sale junto a cada comentario; si no viene, queda vacío.</v>
+      </c>
+      <c r="D16" t="str">
+        <v>A1B2C3D4</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fase 193: Encuesta de Mobilize con la base completa de Wolkvox (v1.81.0)
- La plantilla del Centro es el export HistIVR completo (25 columnas, en
  su orden); las que no se leen van marcadas. Ficha regenerada.
- El lector informa columnas usadas, ignoradas y filas con ID de llamada;
  la vista previa lo muestra.
- ANI, AGENT_DNI y CUSTOMER_ID nunca se leen (regla de la Fase 131).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_ENCUESTA.xlsx
+++ b/server/plantillas/PLANTILLA_ENCUESTA.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:Y1"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -407,49 +407,113 @@
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
     <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="24.83203125" customWidth="1"/>
+    <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="22" max="22" width="14.83203125" customWidth="1"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1"/>
+    <col min="24" max="24" width="15.83203125" customWidth="1"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>AGENT_ID</v>
+      </c>
+      <c r="B1" t="str">
         <v>AGENT_NAME</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
+        <v>AGENT_DNI</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKILL_ID</v>
+      </c>
+      <c r="E1" t="str">
         <v>SKILL_NAME</v>
       </c>
-      <c r="C1" t="str">
+      <c r="F1" t="str">
         <v>DATE</v>
       </c>
-      <c r="D1" t="str">
+      <c r="G1" t="str">
+        <v>CONN_ID</v>
+      </c>
+      <c r="H1" t="str">
+        <v>ANI</v>
+      </c>
+      <c r="I1" t="str">
+        <v>CUSTOMER_ID</v>
+      </c>
+      <c r="J1" t="str">
         <v>Q01</v>
       </c>
-      <c r="E1" t="str">
+      <c r="K1" t="str">
         <v>Q02</v>
       </c>
-      <c r="F1" t="str">
+      <c r="L1" t="str">
         <v>Q03</v>
       </c>
-      <c r="G1" t="str">
+      <c r="M1" t="str">
         <v>Q04</v>
       </c>
-      <c r="H1" t="str">
+      <c r="N1" t="str">
+        <v>Q05</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Q06</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Q07</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Q08</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Q09</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Q10</v>
+      </c>
+      <c r="T1" t="str">
+        <v>VOICE_MESSAGE_DURATION</v>
+      </c>
+      <c r="U1" t="str">
+        <v>TYPE_INTERACTION</v>
+      </c>
+      <c r="V1" t="str">
+        <v>RESULT</v>
+      </c>
+      <c r="W1" t="str">
+        <v>TIME</v>
+      </c>
+      <c r="X1" t="str">
         <v>VOICE_MESSAGE</v>
       </c>
-      <c r="I1" t="str">
-        <v>CONN_ID</v>
+      <c r="Y1" t="str">
+        <v>FEELING</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E32"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -468,7 +532,7 @@
         <v>De dónde sale</v>
       </c>
       <c r="B2" t="str">
-        <v>Wolkvox: Reportes → numeral 4 (hoja "HistIVR&lt;fecha&gt;"). Se sube tal cual: el encabezado puede estar en la fila 2.</v>
+        <v>Wolkvox: Reportes → numeral 4 (hoja "HistIVR&lt;fecha&gt;"), export completo de 25 columnas. Se sube tal cual, sin armar nada a mano: el encabezado se busca en las primeras filas, y el teléfono (ANI), AGENT_DNI y CUSTOMER_ID nunca se leen ni se guardan.</v>
       </c>
     </row>
     <row r="3">
@@ -514,16 +578,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>AGENT_NAME</v>
+        <v>AGENT_ID</v>
       </c>
       <c r="B8" t="str">
-        <v>Sí</v>
+        <v>No</v>
       </c>
       <c r="C8" t="str">
-        <v>Asesor de la llamada encuestada.</v>
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
       </c>
       <c r="D8" t="str">
-        <v>Asesor Ejemplo Uno</v>
+        <v>0000</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -531,16 +595,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SKILL_NAME</v>
+        <v>AGENT_NAME</v>
       </c>
       <c r="B9" t="str">
         <v>Sí</v>
       </c>
       <c r="C9" t="str">
-        <v>Línea o skill.</v>
+        <v>Asesor de la llamada encuestada.</v>
       </c>
       <c r="D9" t="str">
-        <v>SKILL SAC</v>
+        <v>Asesor Ejemplo Uno</v>
       </c>
       <c r="E9" t="str">
         <v/>
@@ -548,16 +612,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>DATE</v>
+        <v>AGENT_DNI</v>
       </c>
       <c r="B10" t="str">
-        <v>Sí</v>
+        <v>No</v>
       </c>
       <c r="C10" t="str">
-        <v>Fecha de la encuesta.</v>
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
       </c>
       <c r="D10" t="str">
-        <v>2026-08-01 10:20</v>
+        <v>0000000000</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -565,16 +629,16 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Q01</v>
+        <v>SKILL_ID</v>
       </c>
       <c r="B11" t="str">
-        <v>Sí</v>
+        <v>No</v>
       </c>
       <c r="C11" t="str">
-        <v>Pregunta 1, de 0 a 10. "-" = sin respuesta.</v>
-      </c>
-      <c r="D11">
-        <v>9</v>
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>101</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -582,16 +646,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Q02</v>
+        <v>SKILL_NAME</v>
       </c>
       <c r="B12" t="str">
         <v>Sí</v>
       </c>
       <c r="C12" t="str">
-        <v>Pregunta 2, de 1 a 5.</v>
-      </c>
-      <c r="D12">
-        <v>5</v>
+        <v>Línea o skill.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>SKILL SAC</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -599,16 +663,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Q03</v>
+        <v>DATE</v>
       </c>
       <c r="B13" t="str">
         <v>Sí</v>
       </c>
       <c r="C13" t="str">
-        <v>Pregunta 3: 1 = Sí, 2 = No (base de One &amp; Done y FCR).</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
+        <v>Fecha de la encuesta.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>2026-08-01 10:20</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -616,16 +680,16 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Q04</v>
+        <v>CONN_ID</v>
       </c>
       <c r="B14" t="str">
-        <v>Sí</v>
+        <v>No</v>
       </c>
       <c r="C14" t="str">
-        <v>Pregunta 4, de 1 a 5.</v>
-      </c>
-      <c r="D14">
-        <v>4</v>
+        <v>ID de la llamada en Wolkvox. Sale junto a cada comentario y en el Excel; si un archivo no lo trae, queda vacío.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>A1B2C3D4</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -633,16 +697,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>VOICE_MESSAGE</v>
+        <v>ANI</v>
       </c>
       <c r="B15" t="str">
         <v>No</v>
       </c>
       <c r="C15" t="str">
-        <v>Comentario (opcional).</v>
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
       </c>
       <c r="D15" t="str">
-        <v>Buena atención</v>
+        <v>3000000001</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -650,24 +714,296 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>CONN_ID</v>
+        <v>CUSTOMER_ID</v>
       </c>
       <c r="B16" t="str">
         <v>No</v>
       </c>
       <c r="C16" t="str">
-        <v>ID de la llamada en Wolkvox (opcional). Sale junto a cada comentario; si no viene, queda vacío.</v>
+        <v>Viene en el export de Wolkvox; el sistema nunca la lee ni la guarda.</v>
       </c>
       <c r="D16" t="str">
-        <v>A1B2C3D4</v>
+        <v>-</v>
       </c>
       <c r="E16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Q01</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Pregunta 1, de 0 a 10. "-" = sin respuesta.</v>
+      </c>
+      <c r="D17">
+        <v>9</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Q02</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Pregunta 2, de 1 a 5.</v>
+      </c>
+      <c r="D18">
+        <v>5</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Q03</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Pregunta 3: 1 = Sí, 2 = No (base de One &amp; Done y FCR).</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Q04</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Pregunta 4, de 1 a 5.</v>
+      </c>
+      <c r="D20">
+        <v>4</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Q05</v>
+      </c>
+      <c r="B21" t="str">
+        <v>No</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>-</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Q06</v>
+      </c>
+      <c r="B22" t="str">
+        <v>No</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>-</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Q07</v>
+      </c>
+      <c r="B23" t="str">
+        <v>No</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>-</v>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Q08</v>
+      </c>
+      <c r="B24" t="str">
+        <v>No</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>-</v>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Q09</v>
+      </c>
+      <c r="B25" t="str">
+        <v>No</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>-</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Q10</v>
+      </c>
+      <c r="B26" t="str">
+        <v>No</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>-</v>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>VOICE_MESSAGE_DURATION</v>
+      </c>
+      <c r="B27" t="str">
+        <v>No</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TYPE_INTERACTION</v>
+      </c>
+      <c r="B28" t="str">
+        <v>No</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D28" t="str">
+        <v>inbound</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>RESULT</v>
+      </c>
+      <c r="B29" t="str">
+        <v>No</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>-</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TIME</v>
+      </c>
+      <c r="B30" t="str">
+        <v>No</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>VOICE_MESSAGE</v>
+      </c>
+      <c r="B31" t="str">
+        <v>No</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Comentario (opcional).</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Buena atención</v>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>FEELING</v>
+      </c>
+      <c r="B32" t="str">
+        <v>No</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+      </c>
+      <c r="D32" t="str">
+        <v>-</v>
+      </c>
+      <c r="E32" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>